<commit_message>
updated subject line in email
</commit_message>
<xml_diff>
--- a/tests/test_cases.xlsx
+++ b/tests/test_cases.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ritin Verma\qa-comparison-agent\tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D50DC55-BFFE-4F6B-B4C2-811942AD2E00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA378018-0973-4AA0-82BF-922C7C9AD4FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -57,10 +57,10 @@
     <t>URL_B</t>
   </si>
   <si>
-    <t>https://www.automationanywhere.com/lp/orchestrating-the-autonomous-enterprise</t>
-  </si>
-  <si>
-    <t>https://acquia-uat.automationanywhere.com/lp/orchestrating-the-autonomous-enterprise?t455raaa</t>
+    <t>https://www.automationanywhere.com/solutions</t>
+  </si>
+  <si>
+    <t>https://acquia-uat.automationanywhere.com/solutions?5tg1s</t>
   </si>
 </sst>
 </file>
@@ -465,9 +465,6 @@
       <c r="B3" s="3"/>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1" xr:uid="{818033B9-6CEA-4C6C-B88C-3DC2FD02C276}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
remove fields from excel
</commit_message>
<xml_diff>
--- a/tests/test_cases.xlsx
+++ b/tests/test_cases.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ritin Verma\qa-comparison-agent\tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA378018-0973-4AA0-82BF-922C7C9AD4FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10B11598-4BAE-4761-BD92-D091A58EE44D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,13 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
-  <si>
-    <t>AUTH_TYPE</t>
-  </si>
-  <si>
-    <t>CREDENTIALS</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>PRIORITY</t>
   </si>
@@ -43,12 +37,6 @@
   </si>
   <si>
     <t>TC1</t>
-  </si>
-  <si>
-    <t>basic</t>
-  </si>
-  <si>
-    <t>uatacquia:tysdduNwIQ1O4</t>
   </si>
   <si>
     <t>URL_A</t>
@@ -410,58 +398,44 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="80.42578125" customWidth="1"/>
     <col min="2" max="2" width="59.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.5703125" customWidth="1"/>
-    <col min="4" max="4" width="25" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.28515625" customWidth="1"/>
-    <col min="6" max="6" width="20.7109375" customWidth="1"/>
+    <col min="3" max="3" width="18.28515625" customWidth="1"/>
+    <col min="4" max="4" width="20.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="D2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D2" t="s">
-        <v>7</v>
-      </c>
-      <c r="E2" t="s">
-        <v>4</v>
-      </c>
-      <c r="F2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B3" s="3"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add email notifications, result history, page health checks
</commit_message>
<xml_diff>
--- a/tests/test_cases.xlsx
+++ b/tests/test_cases.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ritin Verma\qa-comparison-agent\tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10B11598-4BAE-4761-BD92-D091A58EE44D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24C0BAF6-ACE0-40CE-AF70-DF8387433110}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -45,10 +45,10 @@
     <t>URL_B</t>
   </si>
   <si>
-    <t>https://www.automationanywhere.com/solutions</t>
-  </si>
-  <si>
-    <t>https://acquia-uat.automationanywhere.com/solutions?5tg1s</t>
+    <t>https://www.automationanywhere.com/</t>
+  </si>
+  <si>
+    <t>https://acquia-uat.automationanywhere.com/</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Clean up app.py - remove canonical, dotenv, playwright installer
</commit_message>
<xml_diff>
--- a/tests/test_cases.xlsx
+++ b/tests/test_cases.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ritin Verma\qa-comparison-agent\tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24C0BAF6-ACE0-40CE-AF70-DF8387433110}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AC1082C-3FEB-41DB-A615-BCC8E31CCFA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="22">
   <si>
     <t>PRIORITY</t>
   </si>
@@ -33,9 +33,6 @@
     <t>TEST_NAME</t>
   </si>
   <si>
-    <t>high</t>
-  </si>
-  <si>
     <t>TC1</t>
   </si>
   <si>
@@ -45,17 +42,62 @@
     <t>URL_B</t>
   </si>
   <si>
-    <t>https://www.automationanywhere.com/</t>
-  </si>
-  <si>
-    <t>https://acquia-uat.automationanywhere.com/</t>
+    <t>https://acquia-uat.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders?76tybh</t>
+  </si>
+  <si>
+    <t>https://acquia-uat.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders/why-finance-must-automate-now?76tybh</t>
+  </si>
+  <si>
+    <t>https://acquia-uat.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders/use-case-selection-and-prioritization?76tybh</t>
+  </si>
+  <si>
+    <t>https://acquia-uat.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders/best-practices-in-implementing-agentic-execution?76tybh</t>
+  </si>
+  <si>
+    <t>https://acquia-uat.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders/building-the-roi-case?76tybh</t>
+  </si>
+  <si>
+    <t>https://acquia-uat.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders/transformation-defined-by-execution-not-adoption?76tybh</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders </t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders/why-finance-must-automate-now </t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders/use-case-selection-and-prioritization </t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders/best-practices-in-implementing-agentic-execution </t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders/building-the-roi-case </t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders/transformation-defined-by-execution-not-adoption </t>
+  </si>
+  <si>
+    <t>TC2</t>
+  </si>
+  <si>
+    <t>TC3</t>
+  </si>
+  <si>
+    <t>TC4</t>
+  </si>
+  <si>
+    <t>TC5</t>
+  </si>
+  <si>
+    <t>TC6</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -73,6 +115,12 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -398,21 +446,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="80.42578125" customWidth="1"/>
-    <col min="2" max="2" width="59.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="145.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="133.85546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="18.28515625" customWidth="1"/>
     <col min="4" max="4" width="20.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>4</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>5</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>0</v>
@@ -423,22 +471,110 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B3" s="3"/>
+      <c r="B4" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D6" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D7" t="s">
+        <v>21</v>
+      </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="A2" r:id="rId1" tooltip="https://acquia-uat.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders?76tybh" xr:uid="{3D2F392E-126E-4B6F-A082-89F9E49BCC9E}"/>
+    <hyperlink ref="A3" r:id="rId2" tooltip="https://acquia-uat.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders/why-finance-must-automate-now?76tybh" xr:uid="{6FB452B8-017D-4217-8023-F39BB9C4F53D}"/>
+    <hyperlink ref="A4" r:id="rId3" tooltip="https://acquia-uat.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders/use-case-selection-and-prioritization?76tybh" xr:uid="{57ED0B9A-3F3B-43D8-8FC3-BF9B7C54C32A}"/>
+    <hyperlink ref="A5" r:id="rId4" tooltip="https://acquia-uat.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders/best-practices-in-implementing-agentic-execution?76tybh" xr:uid="{072B21A1-0971-46AE-B75A-914F4157F10A}"/>
+    <hyperlink ref="A6" r:id="rId5" tooltip="https://acquia-uat.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders/building-the-roi-case?76tybh" xr:uid="{166B90C2-457E-4D32-BBFF-B53976E1D0C9}"/>
+    <hyperlink ref="A7" r:id="rId6" tooltip="https://acquia-uat.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders/transformation-defined-by-execution-not-adoption?76tybh" xr:uid="{61A9E064-34D2-4ACF-B323-839A52730E62}"/>
+    <hyperlink ref="B2" r:id="rId7" tooltip="https://www.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders" display="https://www.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders" xr:uid="{58F5BA3F-7E71-4EE9-AC37-DD1DE5814AE5}"/>
+    <hyperlink ref="B3" r:id="rId8" tooltip="https://www.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders/why-finance-must-automate-now" display="https://www.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders/why-finance-must-automate-now" xr:uid="{96B67720-C902-4214-A17C-0BDCC352ABD7}"/>
+    <hyperlink ref="B4" r:id="rId9" tooltip="https://www.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders/use-case-selection-and-prioritization" display="https://www.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders/use-case-selection-and-prioritization" xr:uid="{22F6E382-BFF1-4AE0-800E-BDDA244172B3}"/>
+    <hyperlink ref="B5" r:id="rId10" tooltip="https://www.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders/best-practices-in-implementing-agentic-execution" display="https://www.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders/best-practices-in-implementing-agentic-execution" xr:uid="{1EFD2B7F-770F-44A5-B04A-124AEF02C8AB}"/>
+    <hyperlink ref="B6" r:id="rId11" tooltip="https://www.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders/building-the-roi-case" display="https://www.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders/building-the-roi-case" xr:uid="{F286A918-BF93-40F5-B077-5528107721E0}"/>
+    <hyperlink ref="B7" r:id="rId12" tooltip="https://www.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders/transformation-defined-by-execution-not-adoption" display="https://www.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders/transformation-defined-by-execution-not-adoption" xr:uid="{452750E6-9E5A-49BE-905F-08CC7BC887F1}"/>
+    <hyperlink ref="C2" r:id="rId13" tooltip="https://www.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders" display="https://www.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders" xr:uid="{406A5E55-CDC2-4C6F-8524-D016FCE94BC7}"/>
+    <hyperlink ref="C3" r:id="rId14" tooltip="https://www.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders/why-finance-must-automate-now" display="https://www.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders/why-finance-must-automate-now" xr:uid="{BAB567A7-9387-4FB0-BA85-BC786836DD67}"/>
+    <hyperlink ref="C4" r:id="rId15" tooltip="https://www.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders/use-case-selection-and-prioritization" display="https://www.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders/use-case-selection-and-prioritization" xr:uid="{45E54ACC-21DC-4A3B-A377-1C8A465CF461}"/>
+    <hyperlink ref="C5" r:id="rId16" tooltip="https://www.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders/best-practices-in-implementing-agentic-execution" display="https://www.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders/best-practices-in-implementing-agentic-execution" xr:uid="{2DA8DBE1-166C-4BD7-8490-00714720CA4F}"/>
+    <hyperlink ref="C6" r:id="rId17" tooltip="https://www.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders/building-the-roi-case" display="https://www.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders/building-the-roi-case" xr:uid="{BBCA6151-9C83-4710-AE57-873C76A0821B}"/>
+    <hyperlink ref="C7" r:id="rId18" tooltip="https://www.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders/transformation-defined-by-execution-not-adoption" display="https://www.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders/transformation-defined-by-execution-not-adoption" xr:uid="{FE1F742C-40EC-4DF7-9D53-D81BDD62096A}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix SSL warning threshold, remove HTML footer, add sample download
</commit_message>
<xml_diff>
--- a/tests/test_cases.xlsx
+++ b/tests/test_cases.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ritin Verma\qa-comparison-agent\tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AC1082C-3FEB-41DB-A615-BCC8E31CCFA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FB3BDB6-09CE-43B7-8DBC-9DACAF0FD8F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="7">
   <si>
     <t>PRIORITY</t>
   </si>
@@ -42,55 +42,10 @@
     <t>URL_B</t>
   </si>
   <si>
-    <t>https://acquia-uat.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders?76tybh</t>
-  </si>
-  <si>
-    <t>https://acquia-uat.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders/why-finance-must-automate-now?76tybh</t>
-  </si>
-  <si>
-    <t>https://acquia-uat.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders/use-case-selection-and-prioritization?76tybh</t>
-  </si>
-  <si>
-    <t>https://acquia-uat.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders/best-practices-in-implementing-agentic-execution?76tybh</t>
-  </si>
-  <si>
-    <t>https://acquia-uat.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders/building-the-roi-case?76tybh</t>
-  </si>
-  <si>
-    <t>https://acquia-uat.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders/transformation-defined-by-execution-not-adoption?76tybh</t>
-  </si>
-  <si>
     <t xml:space="preserve">https://www.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders </t>
   </si>
   <si>
-    <t xml:space="preserve">https://www.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders/why-finance-must-automate-now </t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders/use-case-selection-and-prioritization </t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders/best-practices-in-implementing-agentic-execution </t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders/building-the-roi-case </t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders/transformation-defined-by-execution-not-adoption </t>
-  </si>
-  <si>
-    <t>TC2</t>
-  </si>
-  <si>
-    <t>TC3</t>
-  </si>
-  <si>
-    <t>TC4</t>
-  </si>
-  <si>
-    <t>TC5</t>
-  </si>
-  <si>
-    <t>TC6</t>
+    <t>P1</t>
   </si>
 </sst>
 </file>
@@ -446,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="145.28515625" bestFit="1" customWidth="1"/>
@@ -474,106 +429,20 @@
         <v>5</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="D2" t="s">
         <v>2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="D3" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D4" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="D5" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="D6" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D7" t="s">
-        <v>21</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1" tooltip="https://acquia-uat.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders?76tybh" xr:uid="{3D2F392E-126E-4B6F-A082-89F9E49BCC9E}"/>
-    <hyperlink ref="A3" r:id="rId2" tooltip="https://acquia-uat.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders/why-finance-must-automate-now?76tybh" xr:uid="{6FB452B8-017D-4217-8023-F39BB9C4F53D}"/>
-    <hyperlink ref="A4" r:id="rId3" tooltip="https://acquia-uat.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders/use-case-selection-and-prioritization?76tybh" xr:uid="{57ED0B9A-3F3B-43D8-8FC3-BF9B7C54C32A}"/>
-    <hyperlink ref="A5" r:id="rId4" tooltip="https://acquia-uat.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders/best-practices-in-implementing-agentic-execution?76tybh" xr:uid="{072B21A1-0971-46AE-B75A-914F4157F10A}"/>
-    <hyperlink ref="A6" r:id="rId5" tooltip="https://acquia-uat.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders/building-the-roi-case?76tybh" xr:uid="{166B90C2-457E-4D32-BBFF-B53976E1D0C9}"/>
-    <hyperlink ref="A7" r:id="rId6" tooltip="https://acquia-uat.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders/transformation-defined-by-execution-not-adoption?76tybh" xr:uid="{61A9E064-34D2-4ACF-B323-839A52730E62}"/>
-    <hyperlink ref="B2" r:id="rId7" tooltip="https://www.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders" display="https://www.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders" xr:uid="{58F5BA3F-7E71-4EE9-AC37-DD1DE5814AE5}"/>
-    <hyperlink ref="B3" r:id="rId8" tooltip="https://www.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders/why-finance-must-automate-now" display="https://www.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders/why-finance-must-automate-now" xr:uid="{96B67720-C902-4214-A17C-0BDCC352ABD7}"/>
-    <hyperlink ref="B4" r:id="rId9" tooltip="https://www.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders/use-case-selection-and-prioritization" display="https://www.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders/use-case-selection-and-prioritization" xr:uid="{22F6E382-BFF1-4AE0-800E-BDDA244172B3}"/>
-    <hyperlink ref="B5" r:id="rId10" tooltip="https://www.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders/best-practices-in-implementing-agentic-execution" display="https://www.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders/best-practices-in-implementing-agentic-execution" xr:uid="{1EFD2B7F-770F-44A5-B04A-124AEF02C8AB}"/>
-    <hyperlink ref="B6" r:id="rId11" tooltip="https://www.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders/building-the-roi-case" display="https://www.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders/building-the-roi-case" xr:uid="{F286A918-BF93-40F5-B077-5528107721E0}"/>
-    <hyperlink ref="B7" r:id="rId12" tooltip="https://www.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders/transformation-defined-by-execution-not-adoption" display="https://www.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders/transformation-defined-by-execution-not-adoption" xr:uid="{452750E6-9E5A-49BE-905F-08CC7BC887F1}"/>
-    <hyperlink ref="C2" r:id="rId13" tooltip="https://www.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders" display="https://www.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders" xr:uid="{406A5E55-CDC2-4C6F-8524-D016FCE94BC7}"/>
-    <hyperlink ref="C3" r:id="rId14" tooltip="https://www.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders/why-finance-must-automate-now" display="https://www.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders/why-finance-must-automate-now" xr:uid="{BAB567A7-9387-4FB0-BA85-BC786836DD67}"/>
-    <hyperlink ref="C4" r:id="rId15" tooltip="https://www.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders/use-case-selection-and-prioritization" display="https://www.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders/use-case-selection-and-prioritization" xr:uid="{45E54ACC-21DC-4A3B-A377-1C8A465CF461}"/>
-    <hyperlink ref="C5" r:id="rId16" tooltip="https://www.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders/best-practices-in-implementing-agentic-execution" display="https://www.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders/best-practices-in-implementing-agentic-execution" xr:uid="{2DA8DBE1-166C-4BD7-8490-00714720CA4F}"/>
-    <hyperlink ref="C6" r:id="rId17" tooltip="https://www.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders/building-the-roi-case" display="https://www.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders/building-the-roi-case" xr:uid="{BBCA6151-9C83-4710-AE57-873C76A0821B}"/>
-    <hyperlink ref="C7" r:id="rId18" tooltip="https://www.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders/transformation-defined-by-execution-not-adoption" display="https://www.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders/transformation-defined-by-execution-not-adoption" xr:uid="{FE1F742C-40EC-4DF7-9D53-D81BDD62096A}"/>
+    <hyperlink ref="B2" r:id="rId1" tooltip="https://www.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders" display="https://www.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders" xr:uid="{58F5BA3F-7E71-4EE9-AC37-DD1DE5814AE5}"/>
+    <hyperlink ref="A2" r:id="rId2" tooltip="https://www.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders" display="https://www.automationanywhere.com/resources/playbook/agentic-ai-for-finance-leaders" xr:uid="{32923CF3-FD2D-436A-93E1-E1968E73A970}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>